<commit_message>
Correct initial area to two rows and three columns
</commit_message>
<xml_diff>
--- a/爱乐之城-五流派数值配置.xlsx
+++ b/爱乐之城-五流派数值配置.xlsx
@@ -2741,7 +2741,7 @@
         <v>initialRows</v>
       </c>
       <c r="B4" t="str">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -2749,7 +2749,7 @@
         <v>initialCols</v>
       </c>
       <c r="B5" t="str">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
Implement V0.3 prop list and five-phase note resolution
</commit_message>
<xml_diff>
--- a/爱乐之城-五流派数值配置.xlsx
+++ b/爱乐之城-五流派数值配置.xlsx
@@ -5,7 +5,8 @@
   <sheets>
     <sheet name="道具" sheetId="1" r:id="rId1"/>
     <sheet name="规则" sheetId="2" r:id="rId2"/>
-    <sheet name="说明" sheetId="3" r:id="rId3"/>
+    <sheet name="版本" sheetId="3" r:id="rId3"/>
+    <sheet name="说明" sheetId="4" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
@@ -498,7 +499,7 @@
         <v>每种加成%</v>
       </c>
       <c r="P2" t="str">
-        <v>相邻其他乐器每有1种，自身基础演奏值增加X%；每次常规出音另产生K个紫色音符，K为相邻其他乐器种类数，最多4。</v>
+        <v>相邻其他乐器每有1种，自身基础演奏值增加X%；每次基础出音时，在第三轮追加K枚紫色四分音符，K为相邻其他乐器种类数，最多4。</v>
       </c>
     </row>
     <row r="3">
@@ -548,7 +549,7 @@
         <v>编组加成%</v>
       </c>
       <c r="P3" t="str">
-        <v>改为每1秒常规产生4K个随机音符，K为场上带“提琴”标签的乐器件数（含自身，最多3）；K达到3时，自身基础演奏值增加X%。</v>
+        <v>基础模版改为每1秒产生4K枚随机品质四分音符，K为场上带提琴标签的乐器件数（含自身，最多3）；K达到3时，自身基础演奏值增加X%。</v>
       </c>
     </row>
     <row r="4">
@@ -598,7 +599,7 @@
         <v>目标加成%</v>
       </c>
       <c r="P4" t="str">
-        <v>场上金色键盘乐器和金色弦乐器的基础演奏值增加X%。</v>
+        <v>场上有至少3种乐器时，金色键盘和金色弦乐器的基础演奏值增加X%。</v>
       </c>
     </row>
     <row r="5">
@@ -677,136 +678,136 @@
         <v>460</v>
       </c>
       <c r="I6">
+        <v>6</v>
+      </c>
+      <c r="J6">
         <v>8</v>
       </c>
-      <c r="J6">
+      <c r="K6">
         <v>10</v>
       </c>
-      <c r="K6">
+      <c r="L6">
         <v>12</v>
       </c>
-      <c r="L6">
+      <c r="M6">
         <v>14</v>
       </c>
-      <c r="M6">
+      <c r="N6">
         <v>16</v>
-      </c>
-      <c r="N6">
-        <v>18</v>
       </c>
       <c r="O6" t="str">
         <v>紫音符加成%</v>
       </c>
       <c r="P6" t="str">
-        <v>自身及相邻乐器产生的紫色音符得分增加X%。</v>
+        <v>场上键盘和弦乐器产生的紫色四分音符得分增加X%。</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>P01</v>
+        <v>B02</v>
       </c>
       <c r="B7" t="str">
-        <v>巡演手风琴</v>
+        <v>小提琴</v>
       </c>
       <c r="C7">
-        <v>960</v>
+        <v>200</v>
       </c>
       <c r="D7">
-        <v>1171</v>
+        <v>244</v>
       </c>
       <c r="E7">
-        <v>1401</v>
+        <v>292</v>
       </c>
       <c r="F7">
-        <v>1651</v>
+        <v>344</v>
       </c>
       <c r="G7">
-        <v>1920</v>
+        <v>400</v>
       </c>
       <c r="H7">
-        <v>2208</v>
+        <v>460</v>
       </c>
       <c r="I7">
-        <v>60</v>
+        <v>3</v>
       </c>
       <c r="J7">
-        <v>66</v>
+        <v>4</v>
       </c>
       <c r="K7">
-        <v>72</v>
+        <v>5</v>
       </c>
       <c r="L7">
-        <v>78</v>
+        <v>6</v>
       </c>
       <c r="M7">
-        <v>84</v>
+        <v>7</v>
       </c>
       <c r="N7">
-        <v>90</v>
+        <v>8</v>
       </c>
       <c r="O7" t="str">
-        <v>复制得分系数%</v>
+        <v>弦乐加成%</v>
       </c>
       <c r="P7" t="str">
-        <v>其他相邻乐器的常规音符经变调后为绿或蓝时，追加1枚同来源、同品质的复制音符；复制音符的基础得分为对应品质基础分的X%。</v>
+        <v>场上弦乐器的基础演奏值增加X%。</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>P02</v>
+        <v>P01</v>
       </c>
       <c r="B8" t="str">
-        <v>民谣吉他</v>
+        <v>巡演手风琴</v>
       </c>
       <c r="C8">
-        <v>500</v>
+        <v>960</v>
       </c>
       <c r="D8">
-        <v>610</v>
+        <v>1171</v>
       </c>
       <c r="E8">
-        <v>730</v>
+        <v>1401</v>
       </c>
       <c r="F8">
-        <v>860</v>
+        <v>1651</v>
       </c>
       <c r="G8">
-        <v>1000</v>
+        <v>1920</v>
       </c>
       <c r="H8">
-        <v>1150</v>
+        <v>2208</v>
       </c>
       <c r="I8">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="J8">
-        <v>28</v>
+        <v>66</v>
       </c>
       <c r="K8">
-        <v>31</v>
+        <v>72</v>
       </c>
       <c r="L8">
-        <v>34</v>
+        <v>78</v>
       </c>
       <c r="M8">
-        <v>37</v>
+        <v>84</v>
       </c>
       <c r="N8">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="O8" t="str">
-        <v>复制概率%</v>
+        <v>复制基础分系数%</v>
       </c>
       <c r="P8" t="str">
-        <v>自身常规音符改按蓝色乐器概率表抽取；其中绿、蓝、紫音符以X%概率追加1枚同品质音符，追加音符按100%品质基础分计。</v>
+        <v>第三轮中，其他键盘和弦乐器剩余的基础绿色、蓝色四分音符各复制1枚；复制保留来源、品质及变调标记，其基础分系数为原音符的X%。</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>P03</v>
+        <v>P02</v>
       </c>
       <c r="B9" t="str">
-        <v>曼陀林</v>
+        <v>尼龙吉他</v>
       </c>
       <c r="C9">
         <v>500</v>
@@ -827,154 +828,154 @@
         <v>1150</v>
       </c>
       <c r="I9">
-        <v>0.2</v>
+        <v>6</v>
       </c>
       <c r="J9">
-        <v>0.24</v>
+        <v>8</v>
       </c>
       <c r="K9">
-        <v>0.28</v>
+        <v>10</v>
       </c>
       <c r="L9">
-        <v>0.32</v>
+        <v>12</v>
       </c>
       <c r="M9">
-        <v>0.36</v>
+        <v>14</v>
       </c>
       <c r="N9">
-        <v>0.4</v>
+        <v>16</v>
       </c>
       <c r="O9" t="str">
-        <v>每枚固定加分</v>
+        <v>蓝音符加成%</v>
       </c>
       <c r="P9" t="str">
-        <v>自身及相邻乐器来源的追加音符，每枚获得X点固定加分。</v>
+        <v>基础模版改为每0.5秒产生2倍自身占格数的蓝色四分音符；自身来源的蓝色四分音符得分增加X%。</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>P04</v>
+        <v>P03</v>
       </c>
       <c r="B10" t="str">
-        <v>陶笛</v>
+        <v>曼陀林</v>
       </c>
       <c r="C10">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="D10">
-        <v>366</v>
+        <v>610</v>
       </c>
       <c r="E10">
-        <v>438</v>
+        <v>730</v>
       </c>
       <c r="F10">
-        <v>516</v>
+        <v>860</v>
       </c>
       <c r="G10">
-        <v>600</v>
+        <v>1000</v>
       </c>
       <c r="H10">
-        <v>690</v>
+        <v>1150</v>
       </c>
       <c r="I10">
-        <v>10</v>
+        <v>0.2</v>
       </c>
       <c r="J10">
-        <v>12</v>
+        <v>0.24</v>
       </c>
       <c r="K10">
-        <v>14</v>
+        <v>0.28</v>
       </c>
       <c r="L10">
-        <v>16</v>
+        <v>0.32</v>
       </c>
       <c r="M10">
-        <v>18</v>
+        <v>0.36</v>
       </c>
       <c r="N10">
-        <v>20</v>
+        <v>0.4</v>
       </c>
       <c r="O10" t="str">
-        <v>低品质加成%</v>
+        <v>低品质追加固定加分</v>
       </c>
       <c r="P10" t="str">
-        <v>自身及相邻乐器产生的绿色、蓝色音符得分增加X%。</v>
+        <v>键盘和弦乐器来源的追加绿色、蓝色四分音符，每枚获得X点固定加分。</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>P05</v>
+        <v>P04</v>
       </c>
       <c r="B11" t="str">
-        <v>手鼓</v>
+        <v>陶笛</v>
       </c>
       <c r="C11">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="D11">
-        <v>244</v>
+        <v>366</v>
       </c>
       <c r="E11">
-        <v>292</v>
+        <v>438</v>
       </c>
       <c r="F11">
-        <v>344</v>
+        <v>516</v>
       </c>
       <c r="G11">
-        <v>400</v>
+        <v>600</v>
       </c>
       <c r="H11">
-        <v>460</v>
+        <v>690</v>
       </c>
       <c r="I11">
+        <v>8</v>
+      </c>
+      <c r="J11">
+        <v>10</v>
+      </c>
+      <c r="K11">
         <v>12</v>
       </c>
-      <c r="J11">
+      <c r="L11">
         <v>14</v>
       </c>
-      <c r="K11">
+      <c r="M11">
         <v>16</v>
       </c>
-      <c r="L11">
+      <c r="N11">
         <v>18</v>
       </c>
-      <c r="M11">
-        <v>20</v>
-      </c>
-      <c r="N11">
-        <v>22</v>
-      </c>
       <c r="O11" t="str">
-        <v>追加加成%</v>
+        <v>低品质加成%</v>
       </c>
       <c r="P11" t="str">
-        <v>相邻弦乐器产生的追加音符得分增加X%。</v>
+        <v>场上键盘和弦乐器来源的绿色、蓝色四分音符得分增加X%。</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>H01</v>
+        <v>P05</v>
       </c>
       <c r="B12" t="str">
-        <v>鎏金竖琴</v>
+        <v>手鼓</v>
       </c>
       <c r="C12">
-        <v>960</v>
+        <v>200</v>
       </c>
       <c r="D12">
-        <v>1171</v>
+        <v>244</v>
       </c>
       <c r="E12">
-        <v>1401</v>
+        <v>292</v>
       </c>
       <c r="F12">
-        <v>1651</v>
+        <v>344</v>
       </c>
       <c r="G12">
-        <v>1920</v>
+        <v>400</v>
       </c>
       <c r="H12">
-        <v>2208</v>
+        <v>460</v>
       </c>
       <c r="I12">
         <v>10</v>
@@ -995,868 +996,868 @@
         <v>20</v>
       </c>
       <c r="O12" t="str">
-        <v>升品音符加成%</v>
+        <v>指定音符加成%</v>
       </c>
       <c r="P12" t="str">
-        <v>自身及相邻乐器每批常规音符中，按批内顺序将最多2枚蓝或紫音符提升1级；由本效果升品的音符得分增加X%。</v>
+        <v>场上弦乐器来源的蓝色四分音符、紫色八分音符得分增加X%。</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>H02</v>
+        <v>B03</v>
       </c>
       <c r="B13" t="str">
-        <v>黑管</v>
+        <v>尤克里里</v>
       </c>
       <c r="C13">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="D13">
-        <v>610</v>
+        <v>244</v>
       </c>
       <c r="E13">
-        <v>730</v>
+        <v>292</v>
       </c>
       <c r="F13">
-        <v>860</v>
+        <v>344</v>
       </c>
       <c r="G13">
-        <v>1000</v>
+        <v>400</v>
       </c>
       <c r="H13">
-        <v>1150</v>
+        <v>460</v>
       </c>
       <c r="I13">
-        <v>50</v>
+        <v>8</v>
       </c>
       <c r="J13">
-        <v>54</v>
+        <v>10</v>
       </c>
       <c r="K13">
-        <v>58</v>
+        <v>12</v>
       </c>
       <c r="L13">
-        <v>62</v>
+        <v>14</v>
       </c>
       <c r="M13">
-        <v>66</v>
+        <v>16</v>
       </c>
       <c r="N13">
-        <v>70</v>
+        <v>18</v>
       </c>
       <c r="O13" t="str">
-        <v>升品概率%</v>
+        <v>指定音符加成%</v>
       </c>
       <c r="P13" t="str">
-        <v>自身及相邻管乐器产生的蓝色音符以X%概率提升为紫色。</v>
+        <v>场上的追加蓝色四分音符，以及全部蓝色八分音符，得分增加X%。</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>H03</v>
+        <v>H01</v>
       </c>
       <c r="B14" t="str">
-        <v>沙龙钢琴</v>
+        <v>鎏金竖琴</v>
       </c>
       <c r="C14">
-        <v>500</v>
+        <v>960</v>
       </c>
       <c r="D14">
-        <v>610</v>
+        <v>1171</v>
       </c>
       <c r="E14">
-        <v>730</v>
+        <v>1401</v>
       </c>
       <c r="F14">
-        <v>860</v>
+        <v>1651</v>
       </c>
       <c r="G14">
-        <v>1000</v>
+        <v>1920</v>
       </c>
       <c r="H14">
-        <v>1150</v>
+        <v>2208</v>
       </c>
       <c r="I14">
-        <v>12</v>
+        <v>60</v>
       </c>
       <c r="J14">
-        <v>15</v>
+        <v>65</v>
       </c>
       <c r="K14">
-        <v>18</v>
+        <v>70</v>
       </c>
       <c r="L14">
-        <v>21</v>
+        <v>75</v>
       </c>
       <c r="M14">
-        <v>24</v>
+        <v>80</v>
       </c>
       <c r="N14">
-        <v>27</v>
+        <v>85</v>
       </c>
       <c r="O14" t="str">
-        <v>华彩乐句加成%</v>
+        <v>交换音符加成%</v>
       </c>
       <c r="P14" t="str">
-        <v>每第4批常规出音，原始品质低于金的音符提升为金；该批音符得分增加X%。</v>
+        <v>第二轮中，将场上弦乐和管乐来源的基础四分音符，每2枚同为蓝色或同为紫色的音符换成1枚高一级的基础四分音符；每批最多交换2组，优先紫色组。原音符被消耗，新音符继承排序靠前者来源，由本效果生成的音符得分增加X%。</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>H04</v>
+        <v>H02</v>
       </c>
       <c r="B15" t="str">
-        <v>银制长笛</v>
+        <v>黑管</v>
       </c>
       <c r="C15">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="D15">
-        <v>366</v>
+        <v>610</v>
       </c>
       <c r="E15">
-        <v>438</v>
+        <v>730</v>
       </c>
       <c r="F15">
-        <v>516</v>
+        <v>860</v>
       </c>
       <c r="G15">
-        <v>600</v>
+        <v>1000</v>
       </c>
       <c r="H15">
-        <v>690</v>
+        <v>1150</v>
       </c>
       <c r="I15">
-        <v>8</v>
+        <v>50</v>
       </c>
       <c r="J15">
-        <v>10</v>
+        <v>54</v>
       </c>
       <c r="K15">
-        <v>12</v>
+        <v>58</v>
       </c>
       <c r="L15">
-        <v>14</v>
+        <v>62</v>
       </c>
       <c r="M15">
-        <v>16</v>
+        <v>66</v>
       </c>
       <c r="N15">
-        <v>18</v>
+        <v>70</v>
       </c>
       <c r="O15" t="str">
-        <v>高品质加成%</v>
+        <v>升品概率%</v>
       </c>
       <c r="P15" t="str">
-        <v>场上管乐器产生的金色、红色音符得分增加X%。</v>
+        <v>第二轮，管乐来源的蓝色基础四分音符有X%概率升为紫色；第四轮，键盘和管乐来源的蓝色追加四分音符有X%概率升为紫色。</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>H05</v>
+        <v>H03</v>
       </c>
       <c r="B16" t="str">
-        <v>钟琴</v>
+        <v>沙龙钢琴</v>
       </c>
       <c r="C16">
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="D16">
-        <v>244</v>
+        <v>610</v>
       </c>
       <c r="E16">
-        <v>292</v>
+        <v>730</v>
       </c>
       <c r="F16">
-        <v>344</v>
+        <v>860</v>
       </c>
       <c r="G16">
-        <v>400</v>
+        <v>1000</v>
       </c>
       <c r="H16">
-        <v>460</v>
+        <v>1150</v>
       </c>
       <c r="I16">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="J16">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="K16">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="L16">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="M16">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="N16">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="O16" t="str">
-        <v>金音符加成%</v>
+        <v>条件升品加成%</v>
       </c>
       <c r="P16" t="str">
-        <v>自身及相邻乐器产生的金色音符得分增加X%。</v>
+        <v>基础音符改按蓝色乐器概率表产生；若本结算批次第一轮的金色四分音符不少于3枚，第二轮将自身最多2枚蓝或紫色基础四分音符升1级，由本效果升品的音符得分增加X%。</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>R01</v>
+        <v>H04</v>
       </c>
       <c r="B17" t="str">
-        <v>架子鼓</v>
+        <v>银制长笛</v>
       </c>
       <c r="C17">
-        <v>960</v>
+        <v>300</v>
       </c>
       <c r="D17">
-        <v>1171</v>
+        <v>366</v>
       </c>
       <c r="E17">
-        <v>1401</v>
+        <v>438</v>
       </c>
       <c r="F17">
-        <v>1651</v>
+        <v>516</v>
       </c>
       <c r="G17">
-        <v>1920</v>
+        <v>600</v>
       </c>
       <c r="H17">
-        <v>2208</v>
+        <v>690</v>
       </c>
       <c r="I17">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="J17">
-        <v>1.1</v>
+        <v>10</v>
       </c>
       <c r="K17">
-        <v>1.2</v>
+        <v>12</v>
       </c>
       <c r="L17">
-        <v>1.3</v>
+        <v>14</v>
       </c>
       <c r="M17">
-        <v>1.4</v>
+        <v>16</v>
       </c>
       <c r="N17">
-        <v>1.5</v>
+        <v>18</v>
       </c>
       <c r="O17" t="str">
-        <v>高潮秒数</v>
+        <v>高品质加成%</v>
       </c>
       <c r="P17" t="str">
-        <v>场上累计产生250枚音符后进入X秒高潮；高潮期间所有乐器常规出音间隔缩短50%。高潮期间暂停积累；全部常规及追加音符在非高潮期间均可计数。</v>
+        <v>场上管乐器来源的金色、红色四分音符得分增加X%。</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>R02</v>
+        <v>H05</v>
       </c>
       <c r="B18" t="str">
-        <v>摇滚吉他</v>
+        <v>钟琴</v>
       </c>
       <c r="C18">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="D18">
-        <v>610</v>
+        <v>244</v>
       </c>
       <c r="E18">
-        <v>730</v>
+        <v>292</v>
       </c>
       <c r="F18">
-        <v>860</v>
+        <v>344</v>
       </c>
       <c r="G18">
-        <v>1000</v>
+        <v>400</v>
       </c>
       <c r="H18">
-        <v>1150</v>
+        <v>460</v>
       </c>
       <c r="I18">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="J18">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="K18">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="L18">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="M18">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="N18">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="O18" t="str">
-        <v>Solo加成%</v>
+        <v>金音符加成%</v>
       </c>
       <c r="P18" t="str">
-        <v>第5秒开始1秒Solo：暂停其他乐器常规出音，自身每0.5秒产生G枚金色音符，G为开场产音乐器占格总数；Solo音符得分增加X%，均记为追加音符。</v>
+        <v>场上的金色四分音符、金色八分音符得分增加X%。</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>R03</v>
+        <v>B01</v>
       </c>
       <c r="B19" t="str">
-        <v>电贝斯</v>
+        <v>巴松管</v>
       </c>
       <c r="C19">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="D19">
-        <v>610</v>
+        <v>244</v>
       </c>
       <c r="E19">
-        <v>730</v>
+        <v>292</v>
       </c>
       <c r="F19">
-        <v>860</v>
+        <v>344</v>
       </c>
       <c r="G19">
-        <v>1000</v>
+        <v>400</v>
       </c>
       <c r="H19">
-        <v>1150</v>
+        <v>460</v>
       </c>
       <c r="I19">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="J19">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="K19">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="L19">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="M19">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="N19">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="O19" t="str">
-        <v>追加加成%</v>
+        <v>键盘加成%</v>
       </c>
       <c r="P19" t="str">
-        <v>自身常规出音间隔改为0.4秒；自身产生的追加音符得分增加X%。</v>
+        <v>场上键盘乐器的基础演奏值增加X%。</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>R04</v>
+        <v>R01</v>
       </c>
       <c r="B20" t="str">
-        <v>便携风琴</v>
+        <v>架子鼓</v>
       </c>
       <c r="C20">
-        <v>300</v>
+        <v>960</v>
       </c>
       <c r="D20">
-        <v>366</v>
+        <v>1171</v>
       </c>
       <c r="E20">
-        <v>438</v>
+        <v>1401</v>
       </c>
       <c r="F20">
-        <v>516</v>
+        <v>1651</v>
       </c>
       <c r="G20">
-        <v>600</v>
+        <v>1920</v>
       </c>
       <c r="H20">
-        <v>690</v>
+        <v>2208</v>
       </c>
       <c r="I20">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J20">
-        <v>8</v>
+        <v>1.1</v>
       </c>
       <c r="K20">
-        <v>10</v>
+        <v>1.2</v>
       </c>
       <c r="L20">
-        <v>12</v>
+        <v>1.3</v>
       </c>
       <c r="M20">
-        <v>14</v>
+        <v>1.4</v>
       </c>
       <c r="N20">
-        <v>16</v>
+        <v>1.5</v>
       </c>
       <c r="O20" t="str">
-        <v>基础加成%</v>
+        <v>高潮秒数</v>
       </c>
       <c r="P20" t="str">
-        <v>自身常规出音改为每1秒产生2倍占格数的音符；自身基础演奏值增加X%。</v>
+        <v>非高潮且非Solo期间，场上累计250枚四分音符后，下一个结算批次进入X秒高潮；高潮期间弦乐和打击乐器的基础出音间隔减半，基础音符改为八分音符。高潮期间暂停积累，超额计数保留。</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>R05</v>
+        <v>R02</v>
       </c>
       <c r="B21" t="str">
-        <v>踩镲</v>
+        <v>摇滚吉他</v>
       </c>
       <c r="C21">
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="D21">
-        <v>244</v>
+        <v>610</v>
       </c>
       <c r="E21">
-        <v>292</v>
+        <v>730</v>
       </c>
       <c r="F21">
-        <v>344</v>
+        <v>860</v>
       </c>
       <c r="G21">
-        <v>400</v>
+        <v>1000</v>
       </c>
       <c r="H21">
-        <v>460</v>
+        <v>1150</v>
       </c>
       <c r="I21">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="J21">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="K21">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="L21">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="M21">
-        <v>5</v>
+        <v>27</v>
       </c>
       <c r="N21">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="O21" t="str">
-        <v>补拍枚数</v>
+        <v>Solo加成%</v>
       </c>
       <c r="P21" t="str">
-        <v>每个完整1秒窗口结束，若场上其他乐器常规音符不足12枚，追加X枚蓝色音符。</v>
+        <v>第5秒开始1秒Solo，其他乐器暂停基础产音；自身每0.25秒产生G枚紫色八分音符，G为开场产音乐器占格总数。Solo音符得分增加X%，属于基础音符，专用间隔不受高潮影响。</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>J01</v>
+        <v>R03</v>
       </c>
       <c r="B22" t="str">
-        <v>次中音萨克斯</v>
+        <v>电贝斯</v>
       </c>
       <c r="C22">
-        <v>960</v>
+        <v>500</v>
       </c>
       <c r="D22">
-        <v>1171</v>
+        <v>610</v>
       </c>
       <c r="E22">
-        <v>1401</v>
+        <v>730</v>
       </c>
       <c r="F22">
-        <v>1651</v>
+        <v>860</v>
       </c>
       <c r="G22">
-        <v>1920</v>
+        <v>1000</v>
       </c>
       <c r="H22">
-        <v>2208</v>
+        <v>1150</v>
       </c>
       <c r="I22">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="J22">
-        <v>62</v>
+        <v>18</v>
       </c>
       <c r="K22">
-        <v>64</v>
+        <v>21</v>
       </c>
       <c r="L22">
-        <v>66</v>
+        <v>24</v>
       </c>
       <c r="M22">
-        <v>68</v>
+        <v>27</v>
       </c>
       <c r="N22">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="O22" t="str">
-        <v>升品方向概率%</v>
+        <v>八分音符加成%</v>
       </c>
       <c r="P22" t="str">
-        <v>自身及相邻乐器的常规音符执行一次变调：X%概率升品1级，其余概率降品1级；达到品质边界时保持边界品质。</v>
+        <v>基础模版改为每0.25秒产生自身占格数枚蓝色音符，常态为四分音符，每枚基础分系数为65%；自身来源的八分音符得分增加X%。</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>J02</v>
+        <v>R04</v>
       </c>
       <c r="B23" t="str">
-        <v>中音萨克斯</v>
+        <v>便携风琴</v>
       </c>
       <c r="C23">
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="D23">
-        <v>610</v>
+        <v>366</v>
       </c>
       <c r="E23">
-        <v>730</v>
+        <v>438</v>
       </c>
       <c r="F23">
-        <v>860</v>
+        <v>516</v>
       </c>
       <c r="G23">
-        <v>1000</v>
+        <v>600</v>
       </c>
       <c r="H23">
-        <v>1150</v>
+        <v>690</v>
       </c>
       <c r="I23">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="J23">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="K23">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="L23">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="M23">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="N23">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="O23" t="str">
-        <v>变调音符加成%</v>
+        <v>声部属性加成%</v>
       </c>
       <c r="P23" t="str">
-        <v>自身常规音符执行一次变调：50%概率升品1级、50%概率降品1级；实际发生变调的自身音符得分增加X%。</v>
+        <v>场上键盘和打击乐器的基础演奏值增加X%。</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>J03</v>
+        <v>R05</v>
       </c>
       <c r="B24" t="str">
-        <v>爵士钢琴</v>
+        <v>踩镲</v>
       </c>
       <c r="C24">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="D24">
-        <v>610</v>
+        <v>244</v>
       </c>
       <c r="E24">
-        <v>730</v>
+        <v>292</v>
       </c>
       <c r="F24">
-        <v>860</v>
+        <v>344</v>
       </c>
       <c r="G24">
-        <v>1000</v>
+        <v>400</v>
       </c>
       <c r="H24">
-        <v>1150</v>
+        <v>460</v>
       </c>
       <c r="I24">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J24">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="K24">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="L24">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="M24">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="N24">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="O24" t="str">
-        <v>每秒伴奏上限</v>
+        <v>蓝音符加成%</v>
       </c>
       <c r="P24" t="str">
-        <v>其他乐器每有1枚常规音符在变调或升品阶段实际改变过品质，自身追加1枚蓝色音符；每个完整1秒窗口最多追加X枚。</v>
+        <v>场上蓝色四分音符、蓝色八分音符得分增加X%。</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>J04</v>
+        <v>B04</v>
       </c>
       <c r="B25" t="str">
-        <v>班卓琴</v>
+        <v>木琴</v>
       </c>
       <c r="C25">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="D25">
-        <v>366</v>
+        <v>244</v>
       </c>
       <c r="E25">
-        <v>438</v>
+        <v>292</v>
       </c>
       <c r="F25">
-        <v>516</v>
+        <v>344</v>
       </c>
       <c r="G25">
-        <v>600</v>
+        <v>400</v>
       </c>
       <c r="H25">
-        <v>690</v>
+        <v>460</v>
       </c>
       <c r="I25">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="J25">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="K25">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="L25">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="M25">
-        <v>36</v>
+        <v>16</v>
       </c>
       <c r="N25">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="O25" t="str">
-        <v>降品补偿%</v>
+        <v>指定音符加成%</v>
       </c>
       <c r="P25" t="str">
-        <v>自身产生的音符在变调阶段发生降品时，该音符得分增加X%。</v>
+        <v>场上实际随机变调过的四分音符、紫色八分音符得分增加X%。</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>J05</v>
+        <v>J01</v>
       </c>
       <c r="B26" t="str">
-        <v>弱音小号</v>
+        <v>次中音萨克斯</v>
       </c>
       <c r="C26">
-        <v>200</v>
+        <v>960</v>
       </c>
       <c r="D26">
-        <v>244</v>
+        <v>1171</v>
       </c>
       <c r="E26">
-        <v>292</v>
+        <v>1401</v>
       </c>
       <c r="F26">
-        <v>344</v>
+        <v>1651</v>
       </c>
       <c r="G26">
-        <v>400</v>
+        <v>1920</v>
       </c>
       <c r="H26">
-        <v>460</v>
+        <v>2208</v>
       </c>
       <c r="I26">
-        <v>15</v>
+        <v>60</v>
       </c>
       <c r="J26">
-        <v>18</v>
+        <v>62</v>
       </c>
       <c r="K26">
-        <v>21</v>
+        <v>64</v>
       </c>
       <c r="L26">
-        <v>24</v>
+        <v>66</v>
       </c>
       <c r="M26">
-        <v>27</v>
+        <v>68</v>
       </c>
       <c r="N26">
-        <v>30</v>
+        <v>70</v>
       </c>
       <c r="O26" t="str">
-        <v>升品加成%</v>
+        <v>变调发生率%</v>
       </c>
       <c r="P26" t="str">
-        <v>自身产生的音符在变调或升品阶段发生升品时，该音符得分增加X%。</v>
+        <v>本结算批次第一轮的四分音符包含至少3种品质时，第二轮场上弦乐和管乐的基础四分音符有X%概率随机变调；触发后等概率升1级或降1级，其余保持不变。</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>B01</v>
+        <v>J02</v>
       </c>
       <c r="B27" t="str">
-        <v>巴松管</v>
+        <v>中音萨克斯</v>
       </c>
       <c r="C27">
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="D27">
-        <v>244</v>
+        <v>610</v>
       </c>
       <c r="E27">
-        <v>292</v>
+        <v>730</v>
       </c>
       <c r="F27">
-        <v>344</v>
+        <v>860</v>
       </c>
       <c r="G27">
-        <v>400</v>
+        <v>1000</v>
       </c>
       <c r="H27">
-        <v>460</v>
+        <v>1150</v>
       </c>
       <c r="I27">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="J27">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="K27">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="L27">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="M27">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="N27">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="O27" t="str">
-        <v>键盘加成%</v>
+        <v>随机变调加成%</v>
       </c>
       <c r="P27" t="str">
-        <v>自身及相邻键盘乐器的基础演奏值增加X%。</v>
+        <v>第二轮，自身基础四分音符执行一次随机变调：50%概率升品1级、50%概率降品1级；自身来源且实际发生随机变调的四分音符得分增加X%。</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>B02</v>
+        <v>J03</v>
       </c>
       <c r="B28" t="str">
-        <v>小提琴</v>
+        <v>爵士钢琴</v>
       </c>
       <c r="C28">
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="D28">
-        <v>244</v>
+        <v>610</v>
       </c>
       <c r="E28">
-        <v>292</v>
+        <v>730</v>
       </c>
       <c r="F28">
-        <v>344</v>
+        <v>860</v>
       </c>
       <c r="G28">
-        <v>400</v>
+        <v>1000</v>
       </c>
       <c r="H28">
-        <v>460</v>
+        <v>1150</v>
       </c>
       <c r="I28">
+        <v>4</v>
+      </c>
+      <c r="J28">
+        <v>4</v>
+      </c>
+      <c r="K28">
+        <v>5</v>
+      </c>
+      <c r="L28">
+        <v>5</v>
+      </c>
+      <c r="M28">
         <v>6</v>
       </c>
-      <c r="J28">
-        <v>8</v>
-      </c>
-      <c r="K28">
-        <v>10</v>
-      </c>
-      <c r="L28">
-        <v>12</v>
-      </c>
-      <c r="M28">
-        <v>14</v>
-      </c>
       <c r="N28">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="O28" t="str">
-        <v>弦乐加成%</v>
+        <v>每秒伴奏上限</v>
       </c>
       <c r="P28" t="str">
-        <v>自身及相邻弦乐器的基础演奏值增加X%。</v>
+        <v>第三轮，其他乐器每有1枚基础四分音符在第二轮实际发生随机变调，自身追加1枚蓝色四分音符；每1秒窗口最多追加X枚。稳定升品不触发本效果。</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>B03</v>
+        <v>J04</v>
       </c>
       <c r="B29" t="str">
-        <v>尤克里里</v>
+        <v>班卓琴</v>
       </c>
       <c r="C29">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="D29">
-        <v>244</v>
+        <v>366</v>
       </c>
       <c r="E29">
-        <v>292</v>
+        <v>438</v>
       </c>
       <c r="F29">
-        <v>344</v>
+        <v>516</v>
       </c>
       <c r="G29">
-        <v>400</v>
+        <v>600</v>
       </c>
       <c r="H29">
-        <v>460</v>
+        <v>690</v>
       </c>
       <c r="I29">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="J29">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="K29">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="L29">
-        <v>14</v>
+        <v>32</v>
       </c>
       <c r="M29">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="N29">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="O29" t="str">
-        <v>蓝追加加成%</v>
+        <v>降品补偿%</v>
       </c>
       <c r="P29" t="str">
-        <v>场上追加产生的蓝色音符得分增加X%。</v>
+        <v>自身来源的四分音符带有实际随机降品标记时，得分增加X%。</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>B04</v>
+        <v>J05</v>
       </c>
       <c r="B30" t="str">
-        <v>木琴</v>
+        <v>弱音小号</v>
       </c>
       <c r="C30">
         <v>200</v>
@@ -1877,28 +1878,28 @@
         <v>460</v>
       </c>
       <c r="I30">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="J30">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="K30">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="L30">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="M30">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="N30">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="O30" t="str">
-        <v>下秒加成%</v>
+        <v>升品加成%</v>
       </c>
       <c r="P30" t="str">
-        <v>每个完整1秒窗口中，场上追加音符达到8枚时，自身下一秒常规音符得分增加X%。</v>
+        <v>自身来源的四分音符实际升过品时，得分增加X%，每枚只加一次。</v>
       </c>
     </row>
     <row r="31">
@@ -1927,28 +1928,28 @@
         <v>460</v>
       </c>
       <c r="I31">
+        <v>8</v>
+      </c>
+      <c r="J31">
         <v>10</v>
       </c>
-      <c r="J31">
+      <c r="K31">
         <v>12</v>
       </c>
-      <c r="K31">
+      <c r="L31">
         <v>14</v>
       </c>
-      <c r="L31">
+      <c r="M31">
         <v>16</v>
       </c>
-      <c r="M31">
+      <c r="N31">
         <v>18</v>
       </c>
-      <c r="N31">
-        <v>20</v>
-      </c>
       <c r="O31" t="str">
-        <v>变色加成%</v>
+        <v>管乐变色加成%</v>
       </c>
       <c r="P31" t="str">
-        <v>自身及相邻管乐器的实际变色音符得分增加X%。</v>
+        <v>场上管乐器来源的四分音符实际改变过品质时，得分增加X%。</v>
       </c>
     </row>
     <row r="32">
@@ -2048,7 +2049,7 @@
         <v>绿音符加成%</v>
       </c>
       <c r="P33" t="str">
-        <v>自身绿色音符得分增加X%。</v>
+        <v>自身来源的绿色四分音符得分增加X%。</v>
       </c>
     </row>
     <row r="34">
@@ -2148,7 +2149,7 @@
         <v>绿音符加成%</v>
       </c>
       <c r="P35" t="str">
-        <v>自身及相邻乐器的绿色音符得分增加X%。</v>
+        <v>场上弦乐器来源的绿色四分音符得分增加X%。</v>
       </c>
     </row>
     <row r="36">
@@ -2298,7 +2299,7 @@
         <v>蓝音符加成%</v>
       </c>
       <c r="P38" t="str">
-        <v>自身蓝色音符得分增加X%。</v>
+        <v>自身来源的蓝色四分音符得分增加X%。</v>
       </c>
     </row>
     <row r="39">
@@ -2445,10 +2446,10 @@
         <v>18</v>
       </c>
       <c r="O41" t="str">
-        <v>自身音符加成%</v>
+        <v>低品质加成%</v>
       </c>
       <c r="P41" t="str">
-        <v>自身音符得分增加X%。</v>
+        <v>自身来源的绿色、蓝色四分音符得分增加X%。</v>
       </c>
     </row>
     <row r="42">
@@ -2477,28 +2478,28 @@
         <v>0</v>
       </c>
       <c r="I42">
+        <v>8</v>
+      </c>
+      <c r="J42">
         <v>10</v>
       </c>
-      <c r="J42">
+      <c r="K42">
         <v>12</v>
       </c>
-      <c r="K42">
+      <c r="L42">
         <v>14</v>
       </c>
-      <c r="L42">
+      <c r="M42">
         <v>16</v>
       </c>
-      <c r="M42">
+      <c r="N42">
         <v>18</v>
-      </c>
-      <c r="N42">
-        <v>20</v>
       </c>
       <c r="O42" t="str">
         <v>区域属性加成%</v>
       </c>
       <c r="P42" t="str">
-        <v>相邻键盘和弦乐器的基础演奏值增加X%。</v>
+        <v>相邻乐器的基础演奏值增加X%。</v>
       </c>
     </row>
     <row r="43">
@@ -2527,28 +2528,28 @@
         <v>0</v>
       </c>
       <c r="I43">
+        <v>15</v>
+      </c>
+      <c r="J43">
         <v>18</v>
       </c>
-      <c r="J43">
+      <c r="K43">
         <v>21</v>
       </c>
-      <c r="K43">
+      <c r="L43">
         <v>24</v>
       </c>
-      <c r="L43">
+      <c r="M43">
         <v>27</v>
       </c>
-      <c r="M43">
+      <c r="N43">
         <v>30</v>
       </c>
-      <c r="N43">
-        <v>33</v>
-      </c>
       <c r="O43" t="str">
-        <v>区域追加加成%</v>
+        <v>区域低品质加成%</v>
       </c>
       <c r="P43" t="str">
-        <v>相邻乐器产生的追加音符得分增加X%。</v>
+        <v>相邻乐器来源的绿色、蓝色音符得分增加X%。</v>
       </c>
     </row>
     <row r="44">
@@ -2577,28 +2578,28 @@
         <v>0</v>
       </c>
       <c r="I44">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J44">
+        <v>12</v>
+      </c>
+      <c r="K44">
+        <v>14</v>
+      </c>
+      <c r="L44">
+        <v>16</v>
+      </c>
+      <c r="M44">
         <v>18</v>
       </c>
-      <c r="K44">
-        <v>21</v>
-      </c>
-      <c r="L44">
-        <v>24</v>
-      </c>
-      <c r="M44">
-        <v>27</v>
-      </c>
       <c r="N44">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="O44" t="str">
-        <v>区域高品质加成%</v>
+        <v>区域中高品质加成%</v>
       </c>
       <c r="P44" t="str">
-        <v>相邻乐器产生的金色、红色音符得分增加X%。</v>
+        <v>相邻乐器来源的紫色、金色、红色音符得分增加X%。</v>
       </c>
     </row>
     <row r="45">
@@ -2627,28 +2628,28 @@
         <v>0</v>
       </c>
       <c r="I45">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="J45">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="K45">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="L45">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="M45">
-        <v>36</v>
+        <v>16</v>
       </c>
       <c r="N45">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="O45" t="str">
-        <v>爆发加成%</v>
+        <v>区域基础音符加成%</v>
       </c>
       <c r="P45" t="str">
-        <v>高潮或Solo期间，相邻乐器产生的音符得分增加X%。</v>
+        <v>相邻乐器来源的基础音符得分增加X%。</v>
       </c>
     </row>
     <row r="46">
@@ -2695,10 +2696,10 @@
         <v>0.4</v>
       </c>
       <c r="O46" t="str">
-        <v>变色固定加分</v>
+        <v>区域追加固定加分</v>
       </c>
       <c r="P46" t="str">
-        <v>相邻乐器产生的音符实际变色时，额外获得X点固定加分。</v>
+        <v>相邻乐器来源的追加音符每枚获得X点固定加分。</v>
       </c>
     </row>
   </sheetData>
@@ -2913,11 +2914,27 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>20260927-notes-v03</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:A5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>09/27五流派候选45件，基础和效果每级独立</v>
+        <v>09/27五流派候选V0.3 45件，基础和效果每级独立</v>
       </c>
     </row>
     <row r="2">

</xml_diff>